<commit_message>
Archive old experimental templates locally and remove from repo (archived in archive_kbob)
</commit_message>
<xml_diff>
--- a/templates/test_files/Strukturvorlage_DataDictionary_KBOB_FM.xlsx
+++ b/templates/test_files/Strukturvorlage_DataDictionary_KBOB_FM.xlsx
@@ -33099,9 +33099,21 @@
       <c r="H13" s="42" t="n"/>
       <c r="I13" s="42" t="n"/>
       <c r="J13" s="42" t="n"/>
-      <c r="K13" s="42" t="n"/>
-      <c r="L13" s="42" t="n"/>
-      <c r="M13" s="39" t="n"/>
+      <c r="K13" s="42" t="inlineStr">
+        <is>
+          <t>nicht klassifiziert</t>
+        </is>
+      </c>
+      <c r="L13" s="42" t="inlineStr">
+        <is>
+          <t>Zugänglich unentgeltlich</t>
+        </is>
+      </c>
+      <c r="M13" s="39" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
       <c r="N13" s="203" t="n"/>
       <c r="O13" s="105" t="n"/>
       <c r="P13" s="54" t="n"/>
@@ -33116,9 +33128,21 @@
       <c r="H14" s="42" t="n"/>
       <c r="I14" s="42" t="n"/>
       <c r="J14" s="42" t="n"/>
-      <c r="K14" s="42" t="n"/>
-      <c r="L14" s="42" t="n"/>
-      <c r="M14" s="39" t="n"/>
+      <c r="K14" s="42" t="inlineStr">
+        <is>
+          <t>nicht klassifiziert</t>
+        </is>
+      </c>
+      <c r="L14" s="42" t="inlineStr">
+        <is>
+          <t>Zugänglich unentgeltlich</t>
+        </is>
+      </c>
+      <c r="M14" s="39" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
       <c r="N14" s="203" t="n"/>
       <c r="O14" s="105" t="n"/>
       <c r="P14" s="54" t="n"/>
@@ -33129,7 +33153,11 @@
       <c r="D15" s="90" t="n"/>
       <c r="E15" s="90" t="n"/>
       <c r="F15" s="90" t="n"/>
-      <c r="G15" s="42" t="n"/>
+      <c r="G15" s="42" t="inlineStr">
+        <is>
+          <t>KBOB DK FM_i14y.csv</t>
+        </is>
+      </c>
       <c r="H15" s="42" t="n"/>
       <c r="I15" s="42" t="n"/>
       <c r="J15" s="42" t="n"/>
@@ -33146,7 +33174,11 @@
       <c r="D16" s="90" t="n"/>
       <c r="E16" s="200" t="n"/>
       <c r="F16" s="200" t="n"/>
-      <c r="G16" s="200" t="n"/>
+      <c r="G16" s="200" t="inlineStr">
+        <is>
+          <t>KBOB DK FM_i14y.csv</t>
+        </is>
+      </c>
       <c r="H16" s="200" t="n"/>
       <c r="I16" s="200" t="n"/>
       <c r="J16" s="200" t="n"/>

</xml_diff>

<commit_message>
Clear ephemeral Documents rows 13-18 in KBOB example
</commit_message>
<xml_diff>
--- a/templates/test_files/Strukturvorlage_DataDictionary_KBOB_FM.xlsx
+++ b/templates/test_files/Strukturvorlage_DataDictionary_KBOB_FM.xlsx
@@ -33236,33 +33236,13 @@
       <c r="D13" s="90" t="n"/>
       <c r="E13" s="90" t="n"/>
       <c r="F13" s="90" t="n"/>
-      <c r="G13" s="42" t="inlineStr">
-        <is>
-          <t>KBOB DK FM_i14y.csv</t>
-        </is>
-      </c>
-      <c r="H13" s="42" t="inlineStr">
-        <is>
-          <t>KBOB DK FM_i14y.csv (DE) (AI)</t>
-        </is>
-      </c>
+      <c r="G13" s="42" t="n"/>
+      <c r="H13" s="42" t="n"/>
       <c r="I13" s="42" t="n"/>
       <c r="J13" s="42" t="n"/>
-      <c r="K13" s="42" t="inlineStr">
-        <is>
-          <t>nicht klassifiziert</t>
-        </is>
-      </c>
-      <c r="L13" s="42" t="inlineStr">
-        <is>
-          <t>Zugänglich unentgeltlich</t>
-        </is>
-      </c>
-      <c r="M13" s="39" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="K13" s="42" t="n"/>
+      <c r="L13" s="42" t="n"/>
+      <c r="M13" s="39" t="n"/>
       <c r="N13" s="203" t="n"/>
       <c r="O13" s="105" t="n"/>
       <c r="P13" s="54" t="n"/>
@@ -33273,33 +33253,13 @@
       <c r="D14" s="90" t="n"/>
       <c r="E14" s="90" t="n"/>
       <c r="F14" s="90" t="n"/>
-      <c r="G14" s="42" t="inlineStr">
-        <is>
-          <t>KBOB DK FM_i14y.csv</t>
-        </is>
-      </c>
-      <c r="H14" s="42" t="inlineStr">
-        <is>
-          <t>KBOB DK FM_i14y.csv (DE) (AI)</t>
-        </is>
-      </c>
+      <c r="G14" s="42" t="n"/>
+      <c r="H14" s="42" t="n"/>
       <c r="I14" s="42" t="n"/>
       <c r="J14" s="42" t="n"/>
-      <c r="K14" s="42" t="inlineStr">
-        <is>
-          <t>nicht klassifiziert</t>
-        </is>
-      </c>
-      <c r="L14" s="42" t="inlineStr">
-        <is>
-          <t>Zugänglich unentgeltlich</t>
-        </is>
-      </c>
-      <c r="M14" s="39" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="K14" s="42" t="n"/>
+      <c r="L14" s="42" t="n"/>
+      <c r="M14" s="39" t="n"/>
       <c r="N14" s="203" t="n"/>
       <c r="O14" s="105" t="n"/>
       <c r="P14" s="54" t="n"/>
@@ -33310,33 +33270,13 @@
       <c r="D15" s="90" t="n"/>
       <c r="E15" s="90" t="n"/>
       <c r="F15" s="90" t="n"/>
-      <c r="G15" s="42" t="inlineStr">
-        <is>
-          <t>KBOB DK FM_i14y.csv</t>
-        </is>
-      </c>
-      <c r="H15" s="42" t="inlineStr">
-        <is>
-          <t>KBOB DK FM_i14y.csv (DE) (AI)</t>
-        </is>
-      </c>
+      <c r="G15" s="42" t="n"/>
+      <c r="H15" s="42" t="n"/>
       <c r="I15" s="42" t="n"/>
       <c r="J15" s="42" t="n"/>
-      <c r="K15" s="42" t="inlineStr">
-        <is>
-          <t>nicht klassifiziert</t>
-        </is>
-      </c>
-      <c r="L15" s="42" t="inlineStr">
-        <is>
-          <t>Zugänglich unentgeltlich</t>
-        </is>
-      </c>
-      <c r="M15" s="39" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="K15" s="42" t="n"/>
+      <c r="L15" s="42" t="n"/>
+      <c r="M15" s="39" t="n"/>
       <c r="N15" s="203" t="n"/>
       <c r="O15" s="105" t="n"/>
       <c r="P15" s="54" t="n"/>
@@ -33347,33 +33287,13 @@
       <c r="D16" s="90" t="n"/>
       <c r="E16" s="200" t="n"/>
       <c r="F16" s="200" t="n"/>
-      <c r="G16" s="200" t="inlineStr">
-        <is>
-          <t>KBOB DK FM_i14y.csv</t>
-        </is>
-      </c>
-      <c r="H16" s="200" t="inlineStr">
-        <is>
-          <t>KBOB DK FM_i14y.csv (DE) (AI)</t>
-        </is>
-      </c>
+      <c r="G16" s="200" t="n"/>
+      <c r="H16" s="200" t="n"/>
       <c r="I16" s="200" t="n"/>
       <c r="J16" s="200" t="n"/>
-      <c r="K16" s="200" t="inlineStr">
-        <is>
-          <t>nicht klassifiziert</t>
-        </is>
-      </c>
-      <c r="L16" s="200" t="inlineStr">
-        <is>
-          <t>Zugänglich unentgeltlich</t>
-        </is>
-      </c>
-      <c r="M16" s="200" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="K16" s="200" t="n"/>
+      <c r="L16" s="200" t="n"/>
+      <c r="M16" s="200" t="n"/>
       <c r="N16" s="201" t="n"/>
       <c r="P16" s="54" t="n"/>
       <c r="Q16" s="54" t="n"/>
@@ -33383,33 +33303,13 @@
       <c r="D17" s="90" t="n"/>
       <c r="E17" s="202" t="n"/>
       <c r="F17" s="202" t="n"/>
-      <c r="G17" s="42" t="inlineStr">
-        <is>
-          <t>KBOB DK FM_i14y.csv</t>
-        </is>
-      </c>
-      <c r="H17" s="42" t="inlineStr">
-        <is>
-          <t>KBOB DK FM_i14y.csv (DE) (AI)</t>
-        </is>
-      </c>
+      <c r="G17" s="42" t="n"/>
+      <c r="H17" s="42" t="n"/>
       <c r="I17" s="42" t="n"/>
       <c r="J17" s="42" t="n"/>
-      <c r="K17" s="42" t="inlineStr">
-        <is>
-          <t>nicht klassifiziert</t>
-        </is>
-      </c>
-      <c r="L17" s="42" t="inlineStr">
-        <is>
-          <t>Zugänglich unentgeltlich</t>
-        </is>
-      </c>
-      <c r="M17" s="39" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="K17" s="42" t="n"/>
+      <c r="L17" s="42" t="n"/>
+      <c r="M17" s="39" t="n"/>
       <c r="N17" s="203" t="n"/>
       <c r="O17" s="105" t="n"/>
       <c r="P17" s="54" t="n"/>
@@ -33420,33 +33320,13 @@
       <c r="D18" s="90" t="n"/>
       <c r="E18" s="90" t="n"/>
       <c r="F18" s="90" t="n"/>
-      <c r="G18" s="42" t="inlineStr">
-        <is>
-          <t>KBOB DK FM_i14y.csv</t>
-        </is>
-      </c>
-      <c r="H18" s="42" t="inlineStr">
-        <is>
-          <t>KBOB DK FM_i14y.csv (DE) (AI)</t>
-        </is>
-      </c>
+      <c r="G18" s="42" t="n"/>
+      <c r="H18" s="42" t="n"/>
       <c r="I18" s="42" t="n"/>
       <c r="J18" s="42" t="n"/>
-      <c r="K18" s="42" t="inlineStr">
-        <is>
-          <t>nicht klassifiziert</t>
-        </is>
-      </c>
-      <c r="L18" s="42" t="inlineStr">
-        <is>
-          <t>Zugänglich unentgeltlich</t>
-        </is>
-      </c>
-      <c r="M18" s="39" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
+      <c r="K18" s="42" t="n"/>
+      <c r="L18" s="42" t="n"/>
+      <c r="M18" s="39" t="n"/>
       <c r="N18" s="203" t="n"/>
       <c r="O18" s="105" t="n"/>
       <c r="P18" s="54" t="n"/>

</xml_diff>